<commit_message>
drop mount from bom
Claude-Session: https://claude.ai/code/session_01RCYT2QSY7BVZDeTyE9KrC4
</commit_message>
<xml_diff>
--- a/bom/bom-prototype.xlsx
+++ b/bom/bom-prototype.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -692,109 +692,39 @@
     </row>
     <row r="13"/>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Mount</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Hose clamp</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Small worm-drive, sized to the pen barrel</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>mini hose clamp 8-12mm</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>Sold in multipacks; super-glued to the back of the XIAO</t>
-        </is>
-      </c>
-    </row>
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Total, everything</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15"/>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Super glue</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Cyanoacrylate</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>super glue gel</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr"/>
-    </row>
-    <row r="17"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Keep metal away from the USB-C end of the XIAO: the BLE antenna lives there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Nothing conductive may touch the exposed pads on the back of the board.</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Total, everything</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Keep metal away from the USB-C end of the XIAO: the BLE antenna lives there.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Nothing conductive may touch the exposed pads on the back of the board.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Leave the BAT pads uncovered if the cell might be added later.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Laptop software (Pure Data, bridge, dashboard) is free and not part of this BOM.</t>
         </is>

</xml_diff>